<commit_message>
Work on notebook/scenarios for testing FeedDist behaviour
</commit_message>
<xml_diff>
--- a/data/scenarios/feed_dist/fix_default_feeddist.xlsx
+++ b/data/scenarios/feed_dist/fix_default_feeddist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\scenarios\feed_dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A6402B-DCA1-41AF-B49A-AE5BB6C17CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CC4238-A9F3-4BA1-B49C-F6A936B4D374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25320" yWindow="2055" windowWidth="25440" windowHeight="15270" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="54">
   <si>
     <t>f_breed</t>
   </si>
@@ -88,9 +88,6 @@
   </si>
   <si>
     <t>max_fat</t>
-  </si>
-  <si>
-    <t>Drop fixed ley silage from rations</t>
   </si>
   <si>
     <t>maize</t>
@@ -565,9 +562,7 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -577,7 +572,7 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -589,12 +584,12 @@
         <v>1</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -606,14 +601,14 @@
         <v>0</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="H5" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
@@ -624,7 +619,7 @@
         <v>6</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
@@ -638,21 +633,21 @@
         <v>6</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
         <v>25</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F10" s="8">
         <v>6.3</v>
@@ -661,18 +656,18 @@
         <v>7.6</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B11" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F11" s="8">
         <v>6.1</v>
@@ -686,7 +681,7 @@
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F12" s="8">
         <v>6.4</v>
@@ -741,13 +736,13 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F18">
         <v>350</v>
@@ -756,7 +751,7 @@
         <v>300</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
@@ -770,12 +765,12 @@
         <v>6</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D21" t="s">
         <v>16</v>
@@ -787,7 +782,7 @@
         <v>100</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -809,13 +804,13 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -829,26 +824,26 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
         <v>34</v>
       </c>
-      <c r="B2" t="s">
-        <v>35</v>
-      </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="11">
-        <f>H2*$K$2</f>
+        <f t="shared" ref="F2:F7" si="0">H2*$K$2</f>
         <v>308</v>
       </c>
       <c r="H2" s="12">
         <v>280</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K2" s="15">
         <v>1.1000000000000001</v>
@@ -856,67 +851,67 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="11">
-        <f>H3*$K$2</f>
+        <f t="shared" si="0"/>
         <v>16940</v>
       </c>
       <c r="H3" s="12">
         <v>15400</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="11">
-        <f>H4*$K$2</f>
+        <f t="shared" si="0"/>
         <v>1650.0000000000002</v>
       </c>
       <c r="H4" s="12">
         <v>1500</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="11">
-        <f>H5*$K$2</f>
+        <f t="shared" si="0"/>
         <v>1.1000000000000001</v>
       </c>
       <c r="H5" s="12">
@@ -925,19 +920,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E6" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="11">
-        <f>H6*$K$2</f>
+        <f t="shared" si="0"/>
         <v>253.00000000000003</v>
       </c>
       <c r="H6" s="12">
@@ -946,19 +941,19 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="11">
-        <f>H7*$K$2</f>
+        <f t="shared" si="0"/>
         <v>1430.0000000000002</v>
       </c>
       <c r="H7" s="12">
@@ -971,19 +966,19 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="11">
-        <f>H9*$K$2</f>
+        <f t="shared" ref="F9:F28" si="1">H9*$K$2</f>
         <v>3707.0000000000005</v>
       </c>
       <c r="H9" s="12">
@@ -992,19 +987,19 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="11">
-        <f>H10*$K$2</f>
+        <f t="shared" si="1"/>
         <v>8052.0000000000009</v>
       </c>
       <c r="H10" s="12">
@@ -1013,19 +1008,19 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>
       </c>
       <c r="F11" s="11">
-        <f>H11*$K$2</f>
+        <f t="shared" si="1"/>
         <v>14795.000000000002</v>
       </c>
       <c r="H11" s="12">
@@ -1034,19 +1029,19 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="11">
-        <f>H12*$K$2</f>
+        <f t="shared" si="1"/>
         <v>26829.000000000004</v>
       </c>
       <c r="H12" s="12">
@@ -1055,19 +1050,19 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
       </c>
       <c r="F13" s="11">
-        <f>H13*$K$2</f>
+        <f t="shared" si="1"/>
         <v>10098</v>
       </c>
       <c r="H13" s="12">
@@ -1076,19 +1071,19 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E14" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="11">
-        <f>H14*$K$2</f>
+        <f t="shared" si="1"/>
         <v>93104.000000000015</v>
       </c>
       <c r="H14" s="12">
@@ -1097,19 +1092,19 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E15" t="s">
         <v>8</v>
       </c>
       <c r="F15" s="11">
-        <f>H15*$K$2</f>
+        <f t="shared" si="1"/>
         <v>219406.00000000003</v>
       </c>
       <c r="H15" s="12">
@@ -1118,19 +1113,19 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
         <v>8</v>
       </c>
       <c r="F16" s="11">
-        <f>H16*$K$2</f>
+        <f t="shared" si="1"/>
         <v>2519</v>
       </c>
       <c r="H16" s="12">
@@ -1139,19 +1134,19 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E17" t="s">
         <v>8</v>
       </c>
       <c r="F17" s="11">
-        <f>H17*$K$2</f>
+        <f t="shared" si="1"/>
         <v>6633.0000000000009</v>
       </c>
       <c r="H17" s="12">
@@ -1160,19 +1155,19 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E18" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="11">
-        <f>H18*$K$2</f>
+        <f t="shared" si="1"/>
         <v>132</v>
       </c>
       <c r="H18" s="12">
@@ -1181,19 +1176,19 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E19" t="s">
         <v>8</v>
       </c>
       <c r="F19" s="11">
-        <f>H19*$K$2</f>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="H19" s="12">
@@ -1202,19 +1197,19 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E20" t="s">
         <v>8</v>
       </c>
       <c r="F20" s="11">
-        <f>H20*$K$2</f>
+        <f t="shared" si="1"/>
         <v>528</v>
       </c>
       <c r="H20" s="12">
@@ -1223,19 +1218,19 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E21" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="11">
-        <f>H21*$K$2</f>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="H21" s="12">
@@ -1244,19 +1239,19 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E22" t="s">
         <v>8</v>
       </c>
       <c r="F22" s="11">
-        <f>H22*$K$2</f>
+        <f t="shared" si="1"/>
         <v>4026.0000000000005</v>
       </c>
       <c r="H22" s="12">
@@ -1265,19 +1260,19 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E23" t="s">
         <v>8</v>
       </c>
       <c r="F23" s="11">
-        <f>H23*$K$2</f>
+        <f t="shared" si="1"/>
         <v>15389.000000000002</v>
       </c>
       <c r="H23" s="12">
@@ -1286,19 +1281,19 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E24" t="s">
         <v>8</v>
       </c>
       <c r="F24" s="11">
-        <f>H24*$K$2</f>
+        <f t="shared" si="1"/>
         <v>3047.0000000000005</v>
       </c>
       <c r="H24" s="12">
@@ -1307,19 +1302,19 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E25" t="s">
         <v>8</v>
       </c>
       <c r="F25" s="11">
-        <f>H25*$K$2</f>
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
       <c r="H25" s="12">
@@ -1328,19 +1323,19 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D26" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E26" t="s">
         <v>8</v>
       </c>
       <c r="F26" s="11">
-        <f>H26*$K$2</f>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="H26" s="12">
@@ -1349,19 +1344,19 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E27" t="s">
         <v>8</v>
       </c>
       <c r="F27" s="11">
-        <f>H27*$K$2</f>
+        <f t="shared" si="1"/>
         <v>77</v>
       </c>
       <c r="H27" s="12">
@@ -1370,19 +1365,19 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E28" t="s">
         <v>8</v>
       </c>
       <c r="F28" s="11">
-        <f>H28*$K$2</f>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
       <c r="H28" s="12">

</xml_diff>

<commit_message>
WIP update feed pars roughages to NorFor data
</commit_message>
<xml_diff>
--- a/data/scenarios/feed_dist/fix_default_feeddist.xlsx
+++ b/data/scenarios/feed_dist/fix_default_feeddist.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\scenarios\feed_dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CC4238-A9F3-4BA1-B49C-F6A936B4D374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EFFE96B-6D3D-46A9-B33A-6519A4884AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="2055" windowWidth="25440" windowHeight="15270" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1410" yWindow="1305" windowWidth="25305" windowHeight="15240" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CattleHerd" sheetId="1" r:id="rId1"/>
     <sheet name="FeedMgmt" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="54">
   <si>
     <t>f_breed</t>
   </si>
@@ -626,12 +626,7 @@
       <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="E9" s="2"/>
       <c r="H9" s="4" t="s">
         <v>28</v>
       </c>
@@ -703,6 +698,9 @@
         <v>6</v>
       </c>
       <c r="F14" s="10"/>
+      <c r="H14" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="T14" s="8"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
@@ -758,12 +756,7 @@
       <c r="E19" s="2"/>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="D20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="E20" s="2"/>
       <c r="H20" s="4" t="s">
         <v>28</v>
       </c>
@@ -793,7 +786,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6C2837F-3CD4-4696-9D11-D33CB5C9516D}">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -1384,6 +1377,9 @@
         <v>30</v>
       </c>
     </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D30" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>